<commit_message>
fixed some typos in the second sheet
</commit_message>
<xml_diff>
--- a/Finalised Tables and Columns with Datatypes.xlsx
+++ b/Finalised Tables and Columns with Datatypes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/swathirao/Documents/GitHub/DBMS-Project/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/CharishmaChandu/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11104DCB-DB16-4243-9776-A634910AD786}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D384B11E-3715-D84B-BAD3-44B6B00AA209}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34200" windowHeight="21380" activeTab="1" xr2:uid="{F7DC7519-519E-5246-AC15-A6134710BE38}"/>
+    <workbookView xWindow="660" yWindow="600" windowWidth="15000" windowHeight="15920" activeTab="1" xr2:uid="{F7DC7519-519E-5246-AC15-A6134710BE38}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="164">
   <si>
     <t xml:space="preserve">Airline </t>
   </si>
@@ -390,9 +390,6 @@
     <t>AirlineNames</t>
   </si>
   <si>
-    <t>AIRLINE_ID</t>
-  </si>
-  <si>
     <t>StateNames</t>
   </si>
   <si>
@@ -502,9 +499,6 @@
   </si>
   <si>
     <t>DISTANCE</t>
-  </si>
-  <si>
-    <t>DLEAY_ID</t>
   </si>
   <si>
     <t>DELAY_ID</t>
@@ -636,12 +630,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -656,6 +644,12 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -995,7 +989,7 @@
   <cols>
     <col min="1" max="1" width="19.5" customWidth="1"/>
     <col min="2" max="2" width="29.1640625" customWidth="1"/>
-    <col min="3" max="3" width="25" customWidth="1"/>
+    <col min="3" max="3" width="32.83203125" customWidth="1"/>
     <col min="4" max="4" width="20.5" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1011,17 +1005,17 @@
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13" t="s">
+      <c r="B3" s="11"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11" t="s">
         <v>3</v>
       </c>
     </row>
@@ -1056,7 +1050,7 @@
       <c r="B8" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D8" t="s">
@@ -1070,7 +1064,7 @@
       <c r="B9" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="4"/>
+      <c r="C9" s="12"/>
       <c r="D9" s="2" t="s">
         <v>5</v>
       </c>
@@ -1347,7 +1341,7 @@
       <c r="A45" t="s">
         <v>51</v>
       </c>
-      <c r="C45" s="5" t="s">
+      <c r="C45" s="13" t="s">
         <v>52</v>
       </c>
       <c r="D45" s="2" t="s">
@@ -1358,7 +1352,7 @@
       <c r="A46" t="s">
         <v>54</v>
       </c>
-      <c r="C46" s="5"/>
+      <c r="C46" s="13"/>
       <c r="D46" s="2" t="s">
         <v>53</v>
       </c>
@@ -1367,7 +1361,7 @@
       <c r="A47" t="s">
         <v>55</v>
       </c>
-      <c r="C47" s="5"/>
+      <c r="C47" s="13"/>
       <c r="D47" s="2" t="s">
         <v>3</v>
       </c>
@@ -1376,7 +1370,7 @@
       <c r="A48" t="s">
         <v>56</v>
       </c>
-      <c r="C48" s="5"/>
+      <c r="C48" s="13"/>
       <c r="D48" s="2" t="s">
         <v>3</v>
       </c>
@@ -1385,7 +1379,7 @@
       <c r="A49" t="s">
         <v>57</v>
       </c>
-      <c r="C49" s="5"/>
+      <c r="C49" s="13"/>
       <c r="D49" s="2" t="s">
         <v>30</v>
       </c>
@@ -1394,7 +1388,7 @@
       <c r="A50" t="s">
         <v>58</v>
       </c>
-      <c r="C50" s="5"/>
+      <c r="C50" s="13"/>
       <c r="D50" s="2" t="s">
         <v>59</v>
       </c>
@@ -1403,7 +1397,7 @@
       <c r="A51" t="s">
         <v>60</v>
       </c>
-      <c r="C51" s="5"/>
+      <c r="C51" s="13"/>
       <c r="D51" s="2" t="s">
         <v>53</v>
       </c>
@@ -1412,7 +1406,7 @@
       <c r="A52" t="s">
         <v>61</v>
       </c>
-      <c r="C52" s="5"/>
+      <c r="C52" s="13"/>
       <c r="D52" s="2" t="s">
         <v>53</v>
       </c>
@@ -1421,7 +1415,7 @@
       <c r="A53" t="s">
         <v>62</v>
       </c>
-      <c r="C53" s="5"/>
+      <c r="C53" s="13"/>
       <c r="D53" s="2" t="s">
         <v>28</v>
       </c>
@@ -1430,7 +1424,7 @@
       <c r="A54" t="s">
         <v>63</v>
       </c>
-      <c r="C54" s="5"/>
+      <c r="C54" s="13"/>
       <c r="D54" s="2" t="s">
         <v>64</v>
       </c>
@@ -1439,7 +1433,7 @@
       <c r="A55" t="s">
         <v>65</v>
       </c>
-      <c r="C55" s="5"/>
+      <c r="C55" s="13"/>
       <c r="D55" s="2" t="s">
         <v>53</v>
       </c>
@@ -1448,7 +1442,7 @@
       <c r="A56" t="s">
         <v>66</v>
       </c>
-      <c r="C56" s="5"/>
+      <c r="C56" s="13"/>
       <c r="D56" s="2" t="s">
         <v>3</v>
       </c>
@@ -1457,7 +1451,7 @@
       <c r="A57" t="s">
         <v>67</v>
       </c>
-      <c r="C57" s="5"/>
+      <c r="C57" s="13"/>
       <c r="D57" s="2" t="s">
         <v>3</v>
       </c>
@@ -1466,7 +1460,7 @@
       <c r="A58" t="s">
         <v>68</v>
       </c>
-      <c r="C58" s="5"/>
+      <c r="C58" s="13"/>
       <c r="D58" s="2" t="s">
         <v>30</v>
       </c>
@@ -1475,7 +1469,7 @@
       <c r="A59" t="s">
         <v>69</v>
       </c>
-      <c r="C59" s="5"/>
+      <c r="C59" s="13"/>
       <c r="D59" s="2" t="s">
         <v>28</v>
       </c>
@@ -1484,7 +1478,7 @@
       <c r="A60" t="s">
         <v>70</v>
       </c>
-      <c r="C60" s="5"/>
+      <c r="C60" s="13"/>
       <c r="D60" s="2" t="s">
         <v>28</v>
       </c>
@@ -1493,7 +1487,7 @@
       <c r="A61" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="C61" s="5"/>
+      <c r="C61" s="13"/>
       <c r="D61" s="2" t="s">
         <v>28</v>
       </c>
@@ -1502,7 +1496,7 @@
       <c r="A62" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="C62" s="5"/>
+      <c r="C62" s="13"/>
       <c r="D62" s="2" t="s">
         <v>73</v>
       </c>
@@ -1511,7 +1505,7 @@
       <c r="A63" t="s">
         <v>74</v>
       </c>
-      <c r="C63" s="5"/>
+      <c r="C63" s="13"/>
       <c r="D63" s="2" t="s">
         <v>73</v>
       </c>
@@ -1520,7 +1514,7 @@
       <c r="A64" t="s">
         <v>75</v>
       </c>
-      <c r="C64" s="5"/>
+      <c r="C64" s="13"/>
       <c r="D64" s="2" t="s">
         <v>73</v>
       </c>
@@ -1529,7 +1523,7 @@
       <c r="A65" t="s">
         <v>76</v>
       </c>
-      <c r="C65" s="5"/>
+      <c r="C65" s="13"/>
       <c r="D65" s="2" t="s">
         <v>3</v>
       </c>
@@ -1538,7 +1532,7 @@
       <c r="A66" t="s">
         <v>77</v>
       </c>
-      <c r="C66" s="5"/>
+      <c r="C66" s="13"/>
       <c r="D66" s="2" t="s">
         <v>3</v>
       </c>
@@ -1703,7 +1697,8 @@
   <dimension ref="A1:G92"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="59" style="11" customWidth="1"/>
+    <col min="2" max="2" width="59" style="9" customWidth="1"/>
+    <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="25.5" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.6640625" customWidth="1"/>
     <col min="7" max="7" width="22.1640625" customWidth="1"/>
@@ -1711,26 +1706,27 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="B1" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>97</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>162</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>1</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="6" t="s">
         <v>106</v>
       </c>
       <c r="E3">
@@ -1738,7 +1734,7 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="7" t="s">
         <v>102</v>
       </c>
       <c r="C4" t="s">
@@ -1746,38 +1742,38 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="7" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="7" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="7" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="7" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="7" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B10" s="9"/>
+      <c r="B10" s="7"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>2</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="8" t="s">
         <v>107</v>
       </c>
       <c r="E11">
@@ -1785,7 +1781,7 @@
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B12" s="11" t="s">
+      <c r="B12" s="9" t="s">
         <v>104</v>
       </c>
       <c r="C12" t="s">
@@ -1793,7 +1789,7 @@
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="9" t="s">
         <v>105</v>
       </c>
     </row>
@@ -1801,7 +1797,7 @@
       <c r="A15">
         <v>3</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="6" t="s">
         <v>112</v>
       </c>
       <c r="E15">
@@ -1809,7 +1805,7 @@
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B16" s="11" t="s">
+      <c r="B16" s="9" t="s">
         <v>108</v>
       </c>
       <c r="C16" t="s">
@@ -1817,17 +1813,17 @@
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B17" s="11" t="s">
+      <c r="B17" s="9" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B18" s="11" t="s">
+      <c r="B18" s="9" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B19" s="11" t="s">
+      <c r="B19" s="9" t="s">
         <v>111</v>
       </c>
       <c r="C19" t="s">
@@ -1838,7 +1834,7 @@
       <c r="A21">
         <v>4</v>
       </c>
-      <c r="B21" s="8" t="s">
+      <c r="B21" s="6" t="s">
         <v>114</v>
       </c>
       <c r="E21">
@@ -1846,24 +1842,24 @@
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B22" s="11" t="s">
+      <c r="B22" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="C22" s="12" t="s">
-        <v>21</v>
+      <c r="C22" s="10" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B23" s="11" t="s">
+      <c r="B23" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="C23" s="12"/>
+      <c r="C23" s="10"/>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>5</v>
       </c>
-      <c r="B25" s="8" t="s">
+      <c r="B25" s="6" t="s">
         <v>115</v>
       </c>
       <c r="E25">
@@ -1871,91 +1867,91 @@
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B26" s="11" t="s">
-        <v>116</v>
-      </c>
-      <c r="C26" s="12" t="s">
-        <v>21</v>
+      <c r="B26" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="C26" s="10" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B27" s="11" t="s">
+      <c r="B27" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="C27" s="12"/>
+      <c r="C27" s="10"/>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>6</v>
       </c>
-      <c r="B29" s="8" t="s">
-        <v>117</v>
+      <c r="B29" s="6" t="s">
+        <v>116</v>
       </c>
       <c r="E29">
         <v>2</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B30" s="9" t="s">
+      <c r="B30" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="C30" s="4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B31" s="9" t="s">
-        <v>118</v>
-      </c>
-      <c r="C31" s="6"/>
+      <c r="B31" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="C31" s="4"/>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>7</v>
       </c>
-      <c r="B33" s="8" t="s">
-        <v>119</v>
+      <c r="B33" s="6" t="s">
+        <v>118</v>
       </c>
       <c r="E33">
         <v>5</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B34" s="11" t="s">
-        <v>120</v>
+      <c r="B34" s="9" t="s">
+        <v>119</v>
       </c>
       <c r="C34" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B35" s="11" t="s">
+      <c r="B35" s="9" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B36" s="9" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B36" s="11" t="s">
-        <v>122</v>
-      </c>
-    </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B37" s="11" t="s">
-        <v>116</v>
+      <c r="B37" s="9" t="s">
+        <v>104</v>
       </c>
       <c r="C37" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B38" s="11" t="s">
-        <v>123</v>
+      <c r="B38" s="9" t="s">
+        <v>122</v>
       </c>
       <c r="C38" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B39" s="11" t="s">
+      <c r="B39" s="9" t="s">
         <v>102</v>
       </c>
       <c r="C39" t="s">
@@ -1963,185 +1959,185 @@
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B40" s="11" t="s">
+      <c r="B40" s="9" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B41" s="9" t="s">
         <v>124</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B41" s="11" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>8</v>
       </c>
-      <c r="B43" s="8" t="s">
-        <v>126</v>
+      <c r="B43" s="6" t="s">
+        <v>125</v>
       </c>
       <c r="E43">
         <v>22</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B44" s="9" t="s">
-        <v>120</v>
-      </c>
-      <c r="C44" s="6" t="s">
+      <c r="B44" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="C44" s="4" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B45" s="9" t="s">
+      <c r="B45" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="C45" s="4"/>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B46" s="7" t="s">
         <v>127</v>
       </c>
-      <c r="C45" s="6"/>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B46" s="9" t="s">
+      <c r="C46" s="4"/>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B47" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="C46" s="6"/>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B47" s="9" t="s">
+      <c r="C47" s="4"/>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B48" s="7" t="s">
         <v>129</v>
       </c>
-      <c r="C47" s="6"/>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B48" s="9" t="s">
+      <c r="C48" s="4"/>
+    </row>
+    <row r="49" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B49" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="C48" s="6"/>
-    </row>
-    <row r="49" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B49" s="9" t="s">
+      <c r="C49" s="4"/>
+    </row>
+    <row r="50" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B50" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="C49" s="6"/>
-    </row>
-    <row r="50" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B50" s="9" t="s">
+      <c r="C50" s="4"/>
+    </row>
+    <row r="51" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B51" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="C50" s="6"/>
-    </row>
-    <row r="51" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B51" s="9" t="s">
+      <c r="C51" s="4"/>
+    </row>
+    <row r="52" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B52" s="7" t="s">
         <v>133</v>
       </c>
-      <c r="C51" s="6"/>
-    </row>
-    <row r="52" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B52" s="9" t="s">
+      <c r="C52" s="4"/>
+    </row>
+    <row r="53" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B53" s="7" t="s">
         <v>134</v>
       </c>
-      <c r="C52" s="6"/>
-    </row>
-    <row r="53" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B53" s="9" t="s">
+      <c r="C53" s="4"/>
+    </row>
+    <row r="54" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B54" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="C53" s="6"/>
-    </row>
-    <row r="54" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B54" s="9" t="s">
+      <c r="C54" s="4"/>
+    </row>
+    <row r="55" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B55" s="7" t="s">
         <v>136</v>
       </c>
-      <c r="C54" s="6"/>
-    </row>
-    <row r="55" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B55" s="9" t="s">
+      <c r="C55" s="4"/>
+    </row>
+    <row r="56" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B56" s="7" t="s">
         <v>137</v>
       </c>
-      <c r="C55" s="6"/>
-    </row>
-    <row r="56" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B56" s="9" t="s">
+      <c r="C56" s="4"/>
+    </row>
+    <row r="57" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B57" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="C56" s="6"/>
-    </row>
-    <row r="57" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B57" s="9" t="s">
+      <c r="C57" s="4"/>
+    </row>
+    <row r="58" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B58" s="7" t="s">
         <v>139</v>
       </c>
-      <c r="C57" s="6"/>
-    </row>
-    <row r="58" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B58" s="9" t="s">
+      <c r="C58" s="4"/>
+    </row>
+    <row r="59" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B59" s="7" t="s">
         <v>140</v>
       </c>
-      <c r="C58" s="6"/>
-    </row>
-    <row r="59" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B59" s="9" t="s">
+      <c r="C59" s="4"/>
+    </row>
+    <row r="60" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B60" s="7" t="s">
         <v>141</v>
       </c>
-      <c r="C59" s="6"/>
-    </row>
-    <row r="60" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B60" s="9" t="s">
+      <c r="C60" s="4"/>
+    </row>
+    <row r="61" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B61" s="7" t="s">
         <v>142</v>
       </c>
-      <c r="C60" s="6"/>
-    </row>
-    <row r="61" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B61" s="9" t="s">
+      <c r="C61" s="4"/>
+    </row>
+    <row r="62" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B62" s="7" t="s">
         <v>143</v>
       </c>
-      <c r="C61" s="6"/>
-    </row>
-    <row r="62" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B62" s="9" t="s">
+      <c r="C62" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="63" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B63" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="C62" s="6" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="63" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B63" s="9" t="s">
+      <c r="C63" s="4"/>
+    </row>
+    <row r="64" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B64" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="C63" s="6"/>
-    </row>
-    <row r="64" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B64" s="9" t="s">
+      <c r="C64" s="4"/>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B65" s="7" t="s">
         <v>146</v>
       </c>
-      <c r="C64" s="6"/>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B65" s="9" t="s">
+      <c r="C65" s="4"/>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B66" s="7" t="s">
         <v>147</v>
       </c>
-      <c r="C65" s="6"/>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B66" s="9" t="s">
+      <c r="C66" s="4"/>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B67" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="C66" s="6"/>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B67" s="9" t="s">
-        <v>149</v>
-      </c>
-      <c r="C67" s="6"/>
+      <c r="C67" s="4"/>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A69">
         <v>9</v>
       </c>
-      <c r="B69" s="8" t="s">
-        <v>150</v>
+      <c r="B69" s="6" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B70" s="11" t="s">
-        <v>123</v>
+      <c r="B70" s="9" t="s">
+        <v>122</v>
       </c>
       <c r="C70" t="s">
         <v>7</v>
@@ -2151,37 +2147,37 @@
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B71" s="11" t="s">
-        <v>151</v>
+      <c r="B71" s="9" t="s">
+        <v>150</v>
       </c>
       <c r="C71" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B72" s="11" t="s">
-        <v>152</v>
+      <c r="B72" s="9" t="s">
+        <v>151</v>
       </c>
       <c r="C72" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B73" s="11" t="s">
-        <v>153</v>
+      <c r="B73" s="9" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A75">
         <v>10</v>
       </c>
-      <c r="B75" s="8" t="s">
+      <c r="B75" s="6" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B76" s="11" t="s">
-        <v>154</v>
+      <c r="B76" s="9" t="s">
+        <v>153</v>
       </c>
       <c r="C76" t="s">
         <v>7</v>
@@ -2191,7 +2187,7 @@
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B77" s="11" t="s">
+      <c r="B77" s="9" t="s">
         <v>113</v>
       </c>
     </row>
@@ -2199,13 +2195,13 @@
       <c r="A79">
         <v>11</v>
       </c>
-      <c r="B79" s="8" t="s">
-        <v>157</v>
+      <c r="B79" s="6" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B80" s="9" t="s">
-        <v>144</v>
+      <c r="B80" s="7" t="s">
+        <v>143</v>
       </c>
       <c r="C80" t="s">
         <v>7</v>
@@ -2215,15 +2211,15 @@
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B81" s="11" t="s">
-        <v>158</v>
+      <c r="B81" s="9" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A83">
         <v>12</v>
       </c>
-      <c r="B83" s="8" t="s">
+      <c r="B83" s="6" t="s">
         <v>82</v>
       </c>
       <c r="E83">
@@ -2231,31 +2227,31 @@
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B84" s="11" t="s">
-        <v>155</v>
-      </c>
-      <c r="C84" s="12" t="s">
-        <v>21</v>
+      <c r="B84" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="C84" s="10" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B85" s="11" t="s">
-        <v>120</v>
-      </c>
-      <c r="C85" s="12" t="s">
-        <v>21</v>
+      <c r="B85" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="C85" s="10" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B86" s="11" t="s">
-        <v>156</v>
+      <c r="B86" s="9" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A88">
         <v>13</v>
       </c>
-      <c r="B88" s="8" t="s">
+      <c r="B88" s="6" t="s">
         <v>91</v>
       </c>
       <c r="E88">
@@ -2263,30 +2259,32 @@
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B89" s="11" t="s">
-        <v>120</v>
-      </c>
-      <c r="C89" s="12" t="s">
-        <v>21</v>
+      <c r="B89" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="C89" s="10" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B90" s="11" t="s">
+      <c r="B90" s="9" t="s">
+        <v>157</v>
+      </c>
+      <c r="C90" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B91" s="9" t="s">
         <v>159</v>
-      </c>
-      <c r="C90" s="12"/>
-    </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B91" s="11" t="s">
-        <v>161</v>
       </c>
       <c r="C91" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B92" s="11" t="s">
-        <v>160</v>
+      <c r="B92" s="9" t="s">
+        <v>158</v>
       </c>
     </row>
   </sheetData>

</xml_diff>